<commit_message>
Implement equipment management features and update generated API client
Replit-Commit-Author: Agent
</commit_message>
<xml_diff>
--- a/بيانات_اختبار_60_تجهيزة.xlsx
+++ b/بيانات_اختبار_60_تجهيزة.xlsx
@@ -4,7 +4,7 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="البيانات" sheetId="1" r:id="rId1"/>
-    <sheet name="التعليمات" sheetId="2" r:id="rId2"/>
+    <sheet name="إحصائيات" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -398,17 +398,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I61"/>
+  <dimension ref="A1:K61"/>
   <cols>
-    <col min="1" max="1" width="36.83203125" customWidth="1"/>
-    <col min="2" max="2" width="22.83203125" customWidth="1"/>
+    <col min="1" max="1" width="42.83203125" customWidth="1"/>
+    <col min="2" max="2" width="20.83203125" customWidth="1"/>
     <col min="3" max="3" width="24.83203125" customWidth="1"/>
-    <col min="4" max="4" width="20.83203125" customWidth="1"/>
+    <col min="4" max="4" width="22.83203125" customWidth="1"/>
     <col min="5" max="5" width="16.83203125" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" customWidth="1"/>
-    <col min="7" max="7" width="18.83203125" customWidth="1"/>
-    <col min="8" max="8" width="26.83203125" customWidth="1"/>
-    <col min="9" max="9" width="44.83203125" customWidth="1"/>
+    <col min="6" max="6" width="10.83203125" customWidth="1"/>
+    <col min="7" max="7" width="20.83203125" customWidth="1"/>
+    <col min="8" max="8" width="12.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="30.83203125" customWidth="1"/>
+    <col min="11" max="11" width="40.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -428,1993 +430,2336 @@
         <v>الحالة</v>
       </c>
       <c r="F1" t="str">
+        <v>الكمية</v>
+      </c>
+      <c r="G1" t="str">
+        <v>الحد الأدنى للكمية</v>
+      </c>
+      <c r="H1" t="str">
         <v>سنة الصنع</v>
       </c>
-      <c r="G1" t="str">
+      <c r="I1" t="str">
         <v>بلد المنشأ</v>
       </c>
-      <c r="H1" t="str">
+      <c r="J1" t="str">
         <v>الحائز الحالي</v>
       </c>
-      <c r="I1" t="str">
+      <c r="K1" t="str">
         <v>ملاحظات</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>جهاز إنعاش قلبي رئوي AED</v>
+        <v>جهاز صدمة كهربائية خارجي آلي (AED)</v>
       </c>
       <c r="B2" t="str">
-        <v>أجهزة الإنعاش</v>
+        <v>جهاز إنعاش</v>
       </c>
       <c r="C2" t="str">
-        <v>Philips HeartStart FRx</v>
+        <v>ZOLL AED Plus</v>
       </c>
       <c r="D2" t="str">
-        <v>SN-AED-001</v>
+        <v>ZL-AED-001</v>
       </c>
       <c r="E2" t="str">
         <v>جيدة</v>
       </c>
       <c r="F2">
-        <v>2022</v>
-      </c>
-      <c r="G2" t="str">
-        <v>هولندا</v>
-      </c>
-      <c r="H2" t="str">
-        <v>مركز الإسعاف المركزي</v>
+        <v>4</v>
+      </c>
+      <c r="G2">
+        <v>2</v>
+      </c>
+      <c r="H2">
+        <v>2021</v>
       </c>
       <c r="I2" t="str">
-        <v>فحص الأقطاب كل 6 أشهر</v>
+        <v>الولايات المتحدة</v>
+      </c>
+      <c r="J2" t="str">
+        <v>سيارة إسعاف 1</v>
+      </c>
+      <c r="K2" t="str">
+        <v>بطارية مكتملة — صيانة دورية سنوية</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>جهاز إنعاش قلبي رئوي AED</v>
+        <v>جهاز صدمة كهربائية خارجي آلي (AED)</v>
       </c>
       <c r="B3" t="str">
-        <v>أجهزة الإنعاش</v>
+        <v>جهاز إنعاش</v>
       </c>
       <c r="C3" t="str">
-        <v>Philips HeartStart FRx</v>
+        <v>ZOLL AED Plus</v>
       </c>
       <c r="D3" t="str">
-        <v>SN-AED-002</v>
+        <v>ZL-AED-002</v>
       </c>
       <c r="E3" t="str">
         <v>جيدة</v>
       </c>
       <c r="F3">
-        <v>2022</v>
-      </c>
-      <c r="G3" t="str">
-        <v>هولندا</v>
-      </c>
-      <c r="H3" t="str">
-        <v>مركز إسعاف المزة</v>
+        <v>4</v>
+      </c>
+      <c r="G3">
+        <v>2</v>
+      </c>
+      <c r="H3">
+        <v>2021</v>
       </c>
       <c r="I3" t="str">
-        <v>وحدتان احتياطيتان — بطارية مشحونة بالكامل</v>
+        <v>الولايات المتحدة</v>
+      </c>
+      <c r="J3" t="str">
+        <v>سيارة إسعاف 2</v>
+      </c>
+      <c r="K3" t="str">
+        <v>بطارية مكتملة</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>جهاز إنعاش قلبي رئوي AED</v>
+        <v>جهاز مراقبة وصدمة كهربائية (Monitor/Defib)</v>
       </c>
       <c r="B4" t="str">
-        <v>أجهزة الإنعاش</v>
+        <v>جهاز إنعاش</v>
       </c>
       <c r="C4" t="str">
-        <v>Zoll AED Plus</v>
+        <v>Philips HeartStart MRx</v>
       </c>
       <c r="D4" t="str">
-        <v>SN-AED-003</v>
+        <v>PH-MRX-2023-01</v>
       </c>
       <c r="E4" t="str">
-        <v>تحتاج فحص</v>
+        <v>جيدة</v>
       </c>
       <c r="F4">
-        <v>2020</v>
-      </c>
-      <c r="G4" t="str">
-        <v>الولايات المتحدة</v>
-      </c>
-      <c r="H4" t="str">
-        <v>مركز إسعاف كفرسوسة</v>
+        <v>2</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="H4">
+        <v>2023</v>
       </c>
       <c r="I4" t="str">
-        <v>آخر فحص قبل 18 شهراً</v>
+        <v>هولندا</v>
+      </c>
+      <c r="J4" t="str">
+        <v>غرفة الطوارئ</v>
+      </c>
+      <c r="K4" t="str">
+        <v>يدعم 12 خيوطاً — معايرة كل 6 أشهر</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>جهاز تنفس اصطناعي محمول</v>
+        <v>جهاز تنفس اصطناعي طارئ (BVM)</v>
       </c>
       <c r="B5" t="str">
-        <v>أجهزة التنفس</v>
+        <v>جهاز تنفس</v>
       </c>
       <c r="C5" t="str">
-        <v>Dräger Oxylog 3000+</v>
+        <v>Ambu SPUR II</v>
       </c>
       <c r="D5" t="str">
-        <v>SN-VENT-001</v>
+        <v/>
       </c>
       <c r="E5" t="str">
         <v>جيدة</v>
       </c>
       <c r="F5">
-        <v>2023</v>
-      </c>
-      <c r="G5" t="str">
-        <v>ألمانيا</v>
-      </c>
-      <c r="H5" t="str">
-        <v>مركز الإسعاف المركزي</v>
+        <v>12</v>
+      </c>
+      <c r="G5">
+        <v>5</v>
+      </c>
+      <c r="H5">
+        <v>2022</v>
       </c>
       <c r="I5" t="str">
-        <v>مع مجموعة كاملة من الأنابيب</v>
+        <v>الدنمارك</v>
+      </c>
+      <c r="J5" t="str">
+        <v>مخزن الطوارئ</v>
+      </c>
+      <c r="K5" t="str">
+        <v>استخدام للبالغين — للاستخدام مرة واحدة</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>جهاز تنفس اصطناعي محمول</v>
+        <v>جهاز تنفس اصطناعي ميكانيكي (Ventilator)</v>
       </c>
       <c r="B6" t="str">
-        <v>أجهزة التنفس</v>
+        <v>جهاز تنفس</v>
       </c>
       <c r="C6" t="str">
-        <v>Dräger Oxylog 3000+</v>
+        <v>Mindray SV300</v>
       </c>
       <c r="D6" t="str">
-        <v>SN-VENT-002</v>
+        <v>MR-SV300-0042</v>
       </c>
       <c r="E6" t="str">
-        <v>في الصيانة</v>
+        <v>جيدة</v>
       </c>
       <c r="F6">
-        <v>2021</v>
-      </c>
-      <c r="G6" t="str">
-        <v>ألمانيا</v>
-      </c>
-      <c r="H6" t="str">
-        <v>ورشة الصيانة</v>
+        <v>3</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6">
+        <v>2020</v>
       </c>
       <c r="I6" t="str">
-        <v>أُرسل للصيانة بسبب خلل في الضغط</v>
+        <v>الصين</v>
+      </c>
+      <c r="J6" t="str">
+        <v>وحدة العناية المركزة</v>
+      </c>
+      <c r="K6" t="str">
+        <v>معايرة أخيرة: يناير 2026</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>جهاز تنفس اصطناعي طارئ</v>
+        <v>جهاز قياس الأكسجين النبضي (Pulse Oximeter)</v>
       </c>
       <c r="B7" t="str">
-        <v>أجهزة التنفس</v>
+        <v>جهاز تشخيص</v>
       </c>
       <c r="C7" t="str">
-        <v>Medumat Standard²</v>
+        <v>Nonin 9590</v>
       </c>
       <c r="D7" t="str">
-        <v>SN-VENT-003</v>
+        <v/>
       </c>
       <c r="E7" t="str">
         <v>جيدة</v>
       </c>
       <c r="F7">
-        <v>2023</v>
-      </c>
-      <c r="G7" t="str">
-        <v>ألمانيا</v>
-      </c>
-      <c r="H7" t="str">
-        <v>مركز إسعاف الميدان</v>
+        <v>15</v>
+      </c>
+      <c r="G7">
+        <v>6</v>
+      </c>
+      <c r="H7">
+        <v>2022</v>
       </c>
       <c r="I7" t="str">
-        <v>طراز مخصص للنقل في سيارات الإسعاف</v>
+        <v>الولايات المتحدة</v>
+      </c>
+      <c r="J7" t="str">
+        <v>مخزن الطوارئ</v>
+      </c>
+      <c r="K7" t="str">
+        <v>محمول — يُوزَّع على السيارات</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>جهاز شفط طبي محمول</v>
+        <v>جهاز شفط إفرازات (Suction Unit)</v>
       </c>
       <c r="B8" t="str">
-        <v>أجهزة الشفط</v>
+        <v>جهاز تنفس</v>
       </c>
       <c r="C8" t="str">
-        <v>Weinmann ACCUVAC Rescue</v>
+        <v>Laerdal Compact</v>
       </c>
       <c r="D8" t="str">
-        <v>SN-SUC-001</v>
+        <v>LAE-SUC-007</v>
       </c>
       <c r="E8" t="str">
         <v>جيدة</v>
       </c>
       <c r="F8">
-        <v>2022</v>
-      </c>
-      <c r="G8" t="str">
-        <v>ألمانيا</v>
-      </c>
-      <c r="H8" t="str">
-        <v>مركز الإسعاف المركزي</v>
+        <v>6</v>
+      </c>
+      <c r="G8">
+        <v>3</v>
+      </c>
+      <c r="H8">
+        <v>2021</v>
       </c>
       <c r="I8" t="str">
-        <v>قوة شفط 300 ملم/زئبق — فلتر بكتيري مدمج</v>
+        <v>النرويج</v>
+      </c>
+      <c r="J8" t="str">
+        <v>سيارة إسعاف 3</v>
+      </c>
+      <c r="K8" t="str">
+        <v>يعمل بالبطارية والكهرباء</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>جهاز شفط طبي محمول</v>
+        <v>جهاز قياس ضغط الدم الرقمي</v>
       </c>
       <c r="B9" t="str">
-        <v>أجهزة الشفط</v>
+        <v>جهاز قياس</v>
       </c>
       <c r="C9" t="str">
-        <v>Laerdal Suction Unit</v>
+        <v>Omron HEM-907</v>
       </c>
       <c r="D9" t="str">
-        <v>SN-SUC-002</v>
+        <v/>
       </c>
       <c r="E9" t="str">
         <v>جيدة</v>
       </c>
       <c r="F9">
-        <v>2021</v>
-      </c>
-      <c r="G9" t="str">
-        <v>النرويج</v>
-      </c>
-      <c r="H9" t="str">
-        <v>مركز إسعاف ركن الدين</v>
+        <v>10</v>
+      </c>
+      <c r="G9">
+        <v>4</v>
+      </c>
+      <c r="H9">
+        <v>2023</v>
       </c>
       <c r="I9" t="str">
-        <v>وحدة احتياطية جاهزة للتشغيل الفوري</v>
+        <v>اليابان</v>
+      </c>
+      <c r="J9" t="str">
+        <v>مخزن الطوارئ</v>
+      </c>
+      <c r="K9" t="str">
+        <v>معايرة كل سنة</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>جهاز شفط طبي محمول</v>
+        <v>جهاز قياس ضغط الدم اليدوي (سفينغومانومتر)</v>
       </c>
       <c r="B10" t="str">
-        <v>أجهزة الشفط</v>
+        <v>جهاز قياس</v>
       </c>
       <c r="C10" t="str">
-        <v>Laerdal Suction Unit</v>
+        <v>Riester Big Ben</v>
       </c>
       <c r="D10" t="str">
-        <v>SN-SUC-003</v>
+        <v/>
       </c>
       <c r="E10" t="str">
-        <v>معطلة</v>
+        <v>جيدة</v>
       </c>
       <c r="F10">
-        <v>2019</v>
-      </c>
-      <c r="G10" t="str">
-        <v>النرويج</v>
-      </c>
-      <c r="H10" t="str">
-        <v>ورشة الصيانة</v>
+        <v>8</v>
+      </c>
+      <c r="G10">
+        <v>3</v>
+      </c>
+      <c r="H10">
+        <v>2022</v>
       </c>
       <c r="I10" t="str">
-        <v>تعطل الموتور - بانتظار قطع الغيار</v>
+        <v>ألمانيا</v>
+      </c>
+      <c r="J10" t="str">
+        <v>مخزن الطوارئ</v>
+      </c>
+      <c r="K10" t="str">
+        <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>منظار حنجرة للتنبيب</v>
+        <v>جهاز رسم القلب (ECG) 12 خيط</v>
       </c>
       <c r="B11" t="str">
-        <v>أجهزة المجرى الهوائي</v>
+        <v>جهاز تشخيص</v>
       </c>
       <c r="C11" t="str">
-        <v>Riester ri-scope L3</v>
+        <v>Schiller AT-102</v>
       </c>
       <c r="D11" t="str">
-        <v>SN-LAR-001</v>
+        <v>SCH-ECG-2022-03</v>
       </c>
       <c r="E11" t="str">
         <v>جيدة</v>
       </c>
       <c r="F11">
+        <v>2</v>
+      </c>
+      <c r="G11">
+        <v>1</v>
+      </c>
+      <c r="H11">
         <v>2022</v>
       </c>
-      <c r="G11" t="str">
-        <v>ألمانيا</v>
-      </c>
-      <c r="H11" t="str">
-        <v>مركز الإسعاف المركزي</v>
-      </c>
       <c r="I11" t="str">
-        <v>مجموعة ريشات 3 مقاسات (صغير/متوسط/كبير)</v>
+        <v>سويسرا</v>
+      </c>
+      <c r="J11" t="str">
+        <v>غرفة الطوارئ</v>
+      </c>
+      <c r="K11" t="str">
+        <v>طباعة فورية — ورق حراري</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>منظار حنجرة للتنبيب</v>
+        <v>جهاز قياس السكر في الدم (Glucometer)</v>
       </c>
       <c r="B12" t="str">
-        <v>أجهزة المجرى الهوائي</v>
+        <v>جهاز قياس</v>
       </c>
       <c r="C12" t="str">
-        <v>Heine Macintosh</v>
+        <v>Accu-Chek Active</v>
       </c>
       <c r="D12" t="str">
-        <v>SN-LAR-002</v>
+        <v/>
       </c>
       <c r="E12" t="str">
         <v>جيدة</v>
       </c>
       <c r="F12">
-        <v>2021</v>
-      </c>
-      <c r="G12" t="str">
+        <v>8</v>
+      </c>
+      <c r="G12">
+        <v>3</v>
+      </c>
+      <c r="H12">
+        <v>2023</v>
+      </c>
+      <c r="I12" t="str">
         <v>ألمانيا</v>
       </c>
-      <c r="H12" t="str">
-        <v>مركز إسعاف المزة</v>
-      </c>
-      <c r="I12" t="str">
-        <v>مجموعة ريشات بديلة مرفقة</v>
+      <c r="J12" t="str">
+        <v>مخزن الطوارئ</v>
+      </c>
+      <c r="K12" t="str">
+        <v>يستلزم شرائط اختبار — راجع مخزون الشرائط</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>جهاز BVM للتنفس الاصطناعي اليدوي</v>
+        <v>جهاز مراقبة المريض متعدد المعاملات</v>
       </c>
       <c r="B13" t="str">
-        <v>أجهزة التنفس</v>
+        <v>جهاز مراقبة</v>
       </c>
       <c r="C13" t="str">
-        <v>Laerdal Silicone</v>
+        <v>Mindray iMEC 8</v>
       </c>
       <c r="D13" t="str">
-        <v>SN-BVM-001</v>
+        <v>MR-IMEC-0021</v>
       </c>
       <c r="E13" t="str">
         <v>جيدة</v>
       </c>
       <c r="F13">
-        <v>2023</v>
-      </c>
-      <c r="G13" t="str">
-        <v>النرويج</v>
-      </c>
-      <c r="H13" t="str">
-        <v>مركز الإسعاف المركزي</v>
+        <v>4</v>
+      </c>
+      <c r="G13">
+        <v>2</v>
+      </c>
+      <c r="H13">
+        <v>2021</v>
       </c>
       <c r="I13" t="str">
-        <v>للبالغين — صمام إيجابي-سلبي مزدوج</v>
+        <v>الصين</v>
+      </c>
+      <c r="J13" t="str">
+        <v>وحدة العناية المركزة</v>
+      </c>
+      <c r="K13" t="str">
+        <v>يقيس: ECG, SpO2, NIBP, Temp, EtCO2</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>جهاز BVM للتنفس الاصطناعي اليدوي</v>
+        <v>جهاز مراقبة المريض متعدد المعاملات</v>
       </c>
       <c r="B14" t="str">
-        <v>أجهزة التنفس</v>
+        <v>جهاز مراقبة</v>
       </c>
       <c r="C14" t="str">
-        <v>Ambu SPUR II</v>
+        <v>Mindray iMEC 8</v>
       </c>
       <c r="D14" t="str">
-        <v>SN-BVM-002</v>
+        <v>MR-IMEC-0022</v>
       </c>
       <c r="E14" t="str">
-        <v>جيدة</v>
+        <v>تحتاج فحص</v>
       </c>
       <c r="F14">
-        <v>2022</v>
-      </c>
-      <c r="G14" t="str">
-        <v>الدنمارك</v>
-      </c>
-      <c r="H14" t="str">
-        <v>مركز إسعاف المزة</v>
+        <v>4</v>
+      </c>
+      <c r="G14">
+        <v>2</v>
+      </c>
+      <c r="H14">
+        <v>2021</v>
       </c>
       <c r="I14" t="str">
-        <v>للأطفال — حجم 450 مل</v>
+        <v>الصين</v>
+      </c>
+      <c r="J14" t="str">
+        <v>مخزن الصيانة</v>
+      </c>
+      <c r="K14" t="str">
+        <v>شاشة بها خلل طفيف — بانتظار قطعة غيار</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>جهاز BVM للتنفس الاصطناعي اليدوي</v>
+        <v>ميزان طبي رقمي</v>
       </c>
       <c r="B15" t="str">
-        <v>أجهزة التنفس</v>
+        <v>جهاز قياس</v>
       </c>
       <c r="C15" t="str">
-        <v>Ambu SPUR II</v>
+        <v>Seca 813</v>
       </c>
       <c r="D15" t="str">
-        <v>SN-BVM-003</v>
+        <v>SC-813-0055</v>
       </c>
       <c r="E15" t="str">
-        <v>تحتاج فحص</v>
+        <v>جيدة</v>
       </c>
       <c r="F15">
+        <v>3</v>
+      </c>
+      <c r="G15">
+        <v>1</v>
+      </c>
+      <c r="H15">
         <v>2020</v>
       </c>
-      <c r="G15" t="str">
-        <v>الدنمارك</v>
-      </c>
-      <c r="H15" t="str">
-        <v>مركز إسعاف كفرسوسة</v>
-      </c>
       <c r="I15" t="str">
-        <v>فحص الصمامات مطلوب</v>
+        <v>ألمانيا</v>
+      </c>
+      <c r="J15" t="str">
+        <v>غرفة الكشف</v>
+      </c>
+      <c r="K15" t="str">
+        <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>جهاز أكسجين محمول مع خزان</v>
+        <v>مقياس حرارة رقمي بالأذن</v>
       </c>
       <c r="B16" t="str">
-        <v>أجهزة الأكسجين</v>
+        <v>جهاز قياس</v>
       </c>
       <c r="C16" t="str">
-        <v>Luxfer G-Size</v>
+        <v>Braun ThermoScan 7</v>
       </c>
       <c r="D16" t="str">
-        <v>SN-OXY-001</v>
+        <v/>
       </c>
       <c r="E16" t="str">
         <v>جيدة</v>
       </c>
       <c r="F16">
-        <v>2021</v>
-      </c>
-      <c r="G16" t="str">
-        <v>المملكة المتحدة</v>
-      </c>
-      <c r="H16" t="str">
-        <v>مركز الإسعاف المركزي</v>
+        <v>10</v>
+      </c>
+      <c r="G16">
+        <v>4</v>
+      </c>
+      <c r="H16">
+        <v>2023</v>
       </c>
       <c r="I16" t="str">
-        <v>فحص صلاحية الأسطوانة 2026</v>
+        <v>ألمانيا</v>
+      </c>
+      <c r="J16" t="str">
+        <v>مخزن الطوارئ</v>
+      </c>
+      <c r="K16" t="str">
+        <v>يستلزم غطاء للمسبار — للاستخدام مرة واحدة</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>جهاز مراقبة المريض المحمول</v>
+        <v>نقالة طبية قابلة للطي</v>
       </c>
       <c r="B17" t="str">
-        <v>أجهزة المراقبة</v>
+        <v>معدات نقل</v>
       </c>
       <c r="C17" t="str">
-        <v>Corpuls 3</v>
+        <v>Ferno Model 35</v>
       </c>
       <c r="D17" t="str">
-        <v>SN-MON-001</v>
+        <v>FER-STR-001</v>
       </c>
       <c r="E17" t="str">
         <v>جيدة</v>
       </c>
       <c r="F17">
-        <v>2023</v>
-      </c>
-      <c r="G17" t="str">
-        <v>ألمانيا</v>
-      </c>
-      <c r="H17" t="str">
-        <v>مركز الإسعاف المركزي</v>
+        <v>6</v>
+      </c>
+      <c r="G17">
+        <v>3</v>
+      </c>
+      <c r="H17">
+        <v>2020</v>
       </c>
       <c r="I17" t="str">
-        <v>ECG 12-lead + SpO2 + NIBP</v>
+        <v>الولايات المتحدة</v>
+      </c>
+      <c r="J17" t="str">
+        <v>سيارة إسعاف 1</v>
+      </c>
+      <c r="K17" t="str">
+        <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>جهاز مراقبة المريض المحمول</v>
+        <v>نقالة طبية قابلة للطي</v>
       </c>
       <c r="B18" t="str">
-        <v>أجهزة المراقبة</v>
+        <v>معدات نقل</v>
       </c>
       <c r="C18" t="str">
-        <v>Corpuls 3</v>
+        <v>Ferno Model 35</v>
       </c>
       <c r="D18" t="str">
-        <v>SN-MON-002</v>
+        <v>FER-STR-002</v>
       </c>
       <c r="E18" t="str">
         <v>جيدة</v>
       </c>
       <c r="F18">
-        <v>2022</v>
-      </c>
-      <c r="G18" t="str">
-        <v>ألمانيا</v>
-      </c>
-      <c r="H18" t="str">
-        <v>مركز إسعاف المزة</v>
+        <v>6</v>
+      </c>
+      <c r="G18">
+        <v>3</v>
+      </c>
+      <c r="H18">
+        <v>2020</v>
       </c>
       <c r="I18" t="str">
-        <v>شاشة 12 بوصة — بطارية 8 ساعات</v>
+        <v>الولايات المتحدة</v>
+      </c>
+      <c r="J18" t="str">
+        <v>سيارة إسعاف 2</v>
+      </c>
+      <c r="K18" t="str">
+        <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>جهاز مراقبة المريض المحمول</v>
+        <v>كرسي نقل مرضى (Wheelchair)</v>
       </c>
       <c r="B19" t="str">
-        <v>أجهزة المراقبة</v>
+        <v>معدات نقل</v>
       </c>
       <c r="C19" t="str">
-        <v>Zoll X Series</v>
+        <v>Drive Medical Cruiser III</v>
       </c>
       <c r="D19" t="str">
-        <v>SN-MON-003</v>
+        <v/>
       </c>
       <c r="E19" t="str">
-        <v>في الصيانة</v>
+        <v>جيدة</v>
       </c>
       <c r="F19">
-        <v>2020</v>
-      </c>
-      <c r="G19" t="str">
-        <v>الولايات المتحدة</v>
-      </c>
-      <c r="H19" t="str">
-        <v>ورشة الصيانة</v>
+        <v>8</v>
+      </c>
+      <c r="G19">
+        <v>3</v>
+      </c>
+      <c r="H19">
+        <v>2021</v>
       </c>
       <c r="I19" t="str">
-        <v>صيانة دورية - عودة خلال أسبوع</v>
+        <v>الولايات المتحدة</v>
+      </c>
+      <c r="J19" t="str">
+        <v>قسم الاستقبال</v>
+      </c>
+      <c r="K19" t="str">
+        <v>فولاذ مقاوم للصدأ</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>جهاز قياس ضغط الدم الرقمي</v>
+        <v>جهاز تثبيت العمود الفقري (Spine Board)</v>
       </c>
       <c r="B20" t="str">
-        <v>أجهزة القياس</v>
+        <v>معدات نقل</v>
       </c>
       <c r="C20" t="str">
-        <v>Omron HEM-7320</v>
+        <v>Ferno XF Spineboard</v>
       </c>
       <c r="D20" t="str">
-        <v>SN-BP-001</v>
+        <v/>
       </c>
       <c r="E20" t="str">
         <v>جيدة</v>
       </c>
       <c r="F20">
+        <v>5</v>
+      </c>
+      <c r="G20">
+        <v>2</v>
+      </c>
+      <c r="H20">
         <v>2022</v>
       </c>
-      <c r="G20" t="str">
-        <v>اليابان</v>
-      </c>
-      <c r="H20" t="str">
-        <v>مركز الإسعاف المركزي</v>
-      </c>
       <c r="I20" t="str">
-        <v>بطارية مشحونة — سُجّل في سجل الصيانة</v>
+        <v>الولايات المتحدة</v>
+      </c>
+      <c r="J20" t="str">
+        <v>مخزن الطوارئ</v>
+      </c>
+      <c r="K20" t="str">
+        <v>مع أحزمة تثبيت 3 نقاط</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>جهاز قياس ضغط الدم الرقمي</v>
+        <v>طوق عنق طبي (Cervical Collar) — مقاسات متعددة</v>
       </c>
       <c r="B21" t="str">
-        <v>أجهزة القياس</v>
+        <v>معدات نقل</v>
       </c>
       <c r="C21" t="str">
-        <v>Omron HEM-7320</v>
+        <v>Laerdal Stifneck Select</v>
       </c>
       <c r="D21" t="str">
-        <v>SN-BP-002</v>
+        <v/>
       </c>
       <c r="E21" t="str">
         <v>جيدة</v>
       </c>
       <c r="F21">
-        <v>2022</v>
-      </c>
-      <c r="G21" t="str">
-        <v>اليابان</v>
-      </c>
-      <c r="H21" t="str">
-        <v>مركز إسعاف المزة</v>
+        <v>20</v>
+      </c>
+      <c r="G21">
+        <v>8</v>
+      </c>
+      <c r="H21">
+        <v>2023</v>
       </c>
       <c r="I21" t="str">
-        <v>مزود بذاكرة لآخر 60 قراءة</v>
+        <v>النرويج</v>
+      </c>
+      <c r="J21" t="str">
+        <v>مخزن الطوارئ</v>
+      </c>
+      <c r="K21" t="str">
+        <v>مجموعة من S/M/L/XL</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>جهاز قياس ضغط الدم الرقمي</v>
+        <v>سرير نقل المرضى الكهربائي</v>
       </c>
       <c r="B22" t="str">
-        <v>أجهزة القياس</v>
+        <v>معدات نقل</v>
       </c>
       <c r="C22" t="str">
-        <v>Welch Allyn Connex</v>
+        <v>Stryker Prime Series</v>
       </c>
       <c r="D22" t="str">
-        <v>SN-BP-003</v>
+        <v>STR-BED-2019-01</v>
       </c>
       <c r="E22" t="str">
         <v>جيدة</v>
       </c>
       <c r="F22">
-        <v>2021</v>
-      </c>
-      <c r="G22" t="str">
-        <v>الولايات المتحدة</v>
-      </c>
-      <c r="H22" t="str">
-        <v>مركز إسعاف كفرسوسة</v>
+        <v>10</v>
+      </c>
+      <c r="G22">
+        <v>4</v>
+      </c>
+      <c r="H22">
+        <v>2019</v>
       </c>
       <c r="I22" t="str">
-        <v>مع سوار قياس للمريض المضطجع</v>
+        <v>الولايات المتحدة</v>
+      </c>
+      <c r="J22" t="str">
+        <v>أجنحة المرضى</v>
+      </c>
+      <c r="K22" t="str">
+        <v>فحص دوري كل 6 أشهر</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>جهاز قياس الأكسجين النبضي</v>
+        <v>سرير نقل المرضى الكهربائي</v>
       </c>
       <c r="B23" t="str">
-        <v>أجهزة القياس</v>
+        <v>معدات نقل</v>
       </c>
       <c r="C23" t="str">
-        <v>Masimo Rad-5</v>
+        <v>Stryker Prime Series</v>
       </c>
       <c r="D23" t="str">
-        <v>SN-SPO-001</v>
+        <v>STR-BED-2019-02</v>
       </c>
       <c r="E23" t="str">
-        <v>جيدة</v>
+        <v>في الصيانة</v>
       </c>
       <c r="F23">
-        <v>2023</v>
-      </c>
-      <c r="G23" t="str">
-        <v>الولايات المتحدة</v>
-      </c>
-      <c r="H23" t="str">
-        <v>مركز الإسعاف المركزي</v>
+        <v>10</v>
+      </c>
+      <c r="G23">
+        <v>4</v>
+      </c>
+      <c r="H23">
+        <v>2019</v>
       </c>
       <c r="I23" t="str">
-        <v>شاشة رقمية كبيرة — صوت إنذار</v>
+        <v>الولايات المتحدة</v>
+      </c>
+      <c r="J23" t="str">
+        <v>ورشة الصيانة</v>
+      </c>
+      <c r="K23" t="str">
+        <v>صيانة دورية — عودة خلال أسبوع</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>جهاز قياس الأكسجين النبضي</v>
+        <v>أسطوانة أكسجين 10 لتر مع منظم ضغط</v>
       </c>
       <c r="B24" t="str">
-        <v>أجهزة القياس</v>
+        <v>معدات أكسجين</v>
       </c>
       <c r="C24" t="str">
-        <v>Nonin 9590</v>
+        <v>Air Liquide Cylinder D</v>
       </c>
       <c r="D24" t="str">
-        <v>SN-SPO-002</v>
+        <v>ALQ-O2-0101</v>
       </c>
       <c r="E24" t="str">
         <v>جيدة</v>
       </c>
       <c r="F24">
+        <v>12</v>
+      </c>
+      <c r="G24">
+        <v>5</v>
+      </c>
+      <c r="H24">
         <v>2022</v>
       </c>
-      <c r="G24" t="str">
-        <v>الولايات المتحدة</v>
-      </c>
-      <c r="H24" t="str">
-        <v>مركز إسعاف ركن الدين</v>
-      </c>
       <c r="I24" t="str">
-        <v>نتائج خلال 5 ثوانٍ — دقة ±2%</v>
+        <v>فرنسا</v>
+      </c>
+      <c r="J24" t="str">
+        <v>سيارة إسعاف 1</v>
+      </c>
+      <c r="K24" t="str">
+        <v>مكتملة الشحن — فحص شهري</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>جهاز قياس الأكسجين النبضي</v>
+        <v>أسطوانة أكسجين 10 لتر مع منظم ضغط</v>
       </c>
       <c r="B25" t="str">
-        <v>أجهزة القياس</v>
+        <v>معدات أكسجين</v>
       </c>
       <c r="C25" t="str">
-        <v>Nonin 9590</v>
+        <v>Air Liquide Cylinder D</v>
       </c>
       <c r="D25" t="str">
-        <v>SN-SPO-003</v>
+        <v>ALQ-O2-0102</v>
       </c>
       <c r="E25" t="str">
-        <v>تحتاج فحص</v>
+        <v>جيدة</v>
       </c>
       <c r="F25">
-        <v>2019</v>
-      </c>
-      <c r="G25" t="str">
-        <v>الولايات المتحدة</v>
-      </c>
-      <c r="H25" t="str">
-        <v>مركز إسعاف الميدان</v>
+        <v>12</v>
+      </c>
+      <c r="G25">
+        <v>5</v>
+      </c>
+      <c r="H25">
+        <v>2022</v>
       </c>
       <c r="I25" t="str">
-        <v>دقة القراءة غير مستقرة</v>
+        <v>فرنسا</v>
+      </c>
+      <c r="J25" t="str">
+        <v>سيارة إسعاف 2</v>
+      </c>
+      <c r="K25" t="str">
+        <v>مكتملة الشحن</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>جهاز تخطيط القلب 12-lead</v>
+        <v>قناع أكسجين مع خرطوم (Non-Rebreather Mask)</v>
       </c>
       <c r="B26" t="str">
-        <v>أجهزة التشخيص</v>
+        <v>معدات أكسجين</v>
       </c>
       <c r="C26" t="str">
-        <v>Schiller AT-102</v>
+        <v>Hudson RCI</v>
       </c>
       <c r="D26" t="str">
-        <v>SN-ECG-001</v>
+        <v/>
       </c>
       <c r="E26" t="str">
         <v>جيدة</v>
       </c>
       <c r="F26">
-        <v>2022</v>
-      </c>
-      <c r="G26" t="str">
-        <v>سويسرا</v>
-      </c>
-      <c r="H26" t="str">
-        <v>مركز الإسعاف المركزي</v>
+        <v>30</v>
+      </c>
+      <c r="G26">
+        <v>10</v>
+      </c>
+      <c r="H26">
+        <v>2024</v>
       </c>
       <c r="I26" t="str">
-        <v>مع برنامج تحليل تلقائي</v>
+        <v>الولايات المتحدة</v>
+      </c>
+      <c r="J26" t="str">
+        <v>مخزن الطوارئ</v>
+      </c>
+      <c r="K26" t="str">
+        <v>للاستخدام مرة واحدة — بالغون</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>ميزان حرارة أذني رقمي</v>
+        <v>منظم تدفق الأكسجين (Flow Regulator)</v>
       </c>
       <c r="B27" t="str">
-        <v>أجهزة القياس</v>
+        <v>معدات أكسجين</v>
       </c>
       <c r="C27" t="str">
-        <v>Braun ThermoScan 7</v>
+        <v>Medline MDS110102</v>
       </c>
       <c r="D27" t="str">
-        <v>SN-TMP-001</v>
+        <v/>
       </c>
       <c r="E27" t="str">
         <v>جيدة</v>
       </c>
       <c r="F27">
-        <v>2023</v>
-      </c>
-      <c r="G27" t="str">
-        <v>ألمانيا</v>
-      </c>
-      <c r="H27" t="str">
-        <v>مركز الإسعاف المركزي</v>
+        <v>8</v>
+      </c>
+      <c r="G27">
+        <v>3</v>
+      </c>
+      <c r="H27">
+        <v>2021</v>
       </c>
       <c r="I27" t="str">
-        <v>ميزان حرارة مزدوج أذن/جبهة</v>
+        <v>الولايات المتحدة</v>
+      </c>
+      <c r="J27" t="str">
+        <v>مخزن الطوارئ</v>
+      </c>
+      <c r="K27" t="str">
+        <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>جهاز قياس جلوكوز الدم</v>
+        <v>جهاز مرطب الأكسجين (Humidifier)</v>
       </c>
       <c r="B28" t="str">
-        <v>أجهزة القياس</v>
+        <v>معدات أكسجين</v>
       </c>
       <c r="C28" t="str">
-        <v>Abbott FreeStyle Optium</v>
+        <v>Fisher &amp; Paykel MR310</v>
       </c>
       <c r="D28" t="str">
-        <v>SN-GLU-001</v>
+        <v>FP-HUM-0033</v>
       </c>
       <c r="E28" t="str">
         <v>جيدة</v>
       </c>
       <c r="F28">
-        <v>2022</v>
-      </c>
-      <c r="G28" t="str">
-        <v>الولايات المتحدة</v>
-      </c>
-      <c r="H28" t="str">
-        <v>مركز الإسعاف المركزي</v>
+        <v>4</v>
+      </c>
+      <c r="G28">
+        <v>2</v>
+      </c>
+      <c r="H28">
+        <v>2020</v>
       </c>
       <c r="I28" t="str">
-        <v>ذاكرة 100 قراءة — خيار البلوتوث</v>
+        <v>نيوزيلندا</v>
+      </c>
+      <c r="J28" t="str">
+        <v>وحدة العناية المركزة</v>
+      </c>
+      <c r="K28" t="str">
+        <v>تعقيم أسبوعي</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>نقالة طوارئ قابلة للطي</v>
+        <v>جهاز تخدير (Anesthesia Machine)</v>
       </c>
       <c r="B29" t="str">
-        <v>معدات النقل</v>
+        <v>جهاز تخدير</v>
       </c>
       <c r="C29" t="str">
-        <v>Ferno Model 35A</v>
+        <v>Drager Perseus A500</v>
       </c>
       <c r="D29" t="str">
-        <v>SN-STR-001</v>
+        <v>DRG-ANES-0007</v>
       </c>
       <c r="E29" t="str">
         <v>جيدة</v>
       </c>
       <c r="F29">
-        <v>2022</v>
-      </c>
-      <c r="G29" t="str">
-        <v>الولايات المتحدة</v>
-      </c>
-      <c r="H29" t="str">
-        <v>مركز الإسعاف المركزي</v>
+        <v>2</v>
+      </c>
+      <c r="G29">
+        <v>1</v>
+      </c>
+      <c r="H29">
+        <v>2021</v>
       </c>
       <c r="I29" t="str">
-        <v>حمولة 200 كغ</v>
+        <v>ألمانيا</v>
+      </c>
+      <c r="J29" t="str">
+        <v>غرفة العمليات 1</v>
+      </c>
+      <c r="K29" t="str">
+        <v>معايرة سنوية — آخرها مارس 2026</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>نقالة طوارئ قابلة للطي</v>
+        <v>جهاز تخدير (Anesthesia Machine)</v>
       </c>
       <c r="B30" t="str">
-        <v>معدات النقل</v>
+        <v>جهاز تخدير</v>
       </c>
       <c r="C30" t="str">
-        <v>Ferno Model 35A</v>
+        <v>Drager Fabius GS</v>
       </c>
       <c r="D30" t="str">
-        <v>SN-STR-002</v>
+        <v>DRG-ANES-0008</v>
       </c>
       <c r="E30" t="str">
         <v>جيدة</v>
       </c>
       <c r="F30">
-        <v>2021</v>
-      </c>
-      <c r="G30" t="str">
-        <v>الولايات المتحدة</v>
-      </c>
-      <c r="H30" t="str">
-        <v>مركز إسعاف المزة</v>
+        <v>2</v>
+      </c>
+      <c r="G30">
+        <v>1</v>
+      </c>
+      <c r="H30">
+        <v>2019</v>
       </c>
       <c r="I30" t="str">
-        <v>مع 4 أحزمة ثبيت قابلة للغسيل</v>
+        <v>ألمانيا</v>
+      </c>
+      <c r="J30" t="str">
+        <v>غرفة العمليات 2</v>
+      </c>
+      <c r="K30" t="str">
+        <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>نقالة طوارئ قابلة للطي</v>
+        <v>مضخة حقن وريدي (Infusion Pump)</v>
       </c>
       <c r="B31" t="str">
-        <v>معدات النقل</v>
+        <v>جهاز علاجي</v>
       </c>
       <c r="C31" t="str">
-        <v>Spencer Xtend</v>
+        <v>Baxter Sigma Spectrum</v>
       </c>
       <c r="D31" t="str">
-        <v>SN-STR-003</v>
+        <v>BAX-INF-0201</v>
       </c>
       <c r="E31" t="str">
-        <v>في الصيانة</v>
+        <v>جيدة</v>
       </c>
       <c r="F31">
-        <v>2019</v>
-      </c>
-      <c r="G31" t="str">
-        <v>إيطاليا</v>
-      </c>
-      <c r="H31" t="str">
-        <v>ورشة الصيانة</v>
+        <v>8</v>
+      </c>
+      <c r="G31">
+        <v>3</v>
+      </c>
+      <c r="H31">
+        <v>2022</v>
       </c>
       <c r="I31" t="str">
-        <v>استبدال عجلات</v>
+        <v>الولايات المتحدة</v>
+      </c>
+      <c r="J31" t="str">
+        <v>أجنحة المرضى</v>
+      </c>
+      <c r="K31" t="str">
+        <v>برمجة جرعات مسبقة مُحدَّثة</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>كرسي الدرج للطوارئ</v>
+        <v>مضخة حقن وريدي (Infusion Pump)</v>
       </c>
       <c r="B32" t="str">
-        <v>معدات النقل</v>
+        <v>جهاز علاجي</v>
       </c>
       <c r="C32" t="str">
-        <v>Ferno Stair Chair 40-STX</v>
+        <v>Baxter Sigma Spectrum</v>
       </c>
       <c r="D32" t="str">
-        <v>SN-CHR-001</v>
+        <v>BAX-INF-0202</v>
       </c>
       <c r="E32" t="str">
-        <v>جيدة</v>
+        <v>معطلة</v>
       </c>
       <c r="F32">
+        <v>8</v>
+      </c>
+      <c r="G32">
+        <v>3</v>
+      </c>
+      <c r="H32">
         <v>2022</v>
       </c>
-      <c r="G32" t="str">
-        <v>الولايات المتحدة</v>
-      </c>
-      <c r="H32" t="str">
-        <v>مركز الإسعاف المركزي</v>
-      </c>
       <c r="I32" t="str">
-        <v>قابل للطي في 3 ثوانٍ — خفيف الوزن</v>
+        <v>الولايات المتحدة</v>
+      </c>
+      <c r="J32" t="str">
+        <v>مخزن الصيانة</v>
+      </c>
+      <c r="K32" t="str">
+        <v>خلل في المحرك — بانتظار قطعة غيار</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>كرسي الدرج للطوارئ</v>
+        <v>مضخة حقن وريدي (Syringe Pump)</v>
       </c>
       <c r="B33" t="str">
-        <v>معدات النقل</v>
+        <v>جهاز علاجي</v>
       </c>
       <c r="C33" t="str">
-        <v>Ferno Stair Chair 40-STX</v>
+        <v>Fresenius Kabi Injectomat</v>
       </c>
       <c r="D33" t="str">
-        <v>SN-CHR-002</v>
+        <v>FRK-SYR-0051</v>
       </c>
       <c r="E33" t="str">
         <v>جيدة</v>
       </c>
       <c r="F33">
+        <v>10</v>
+      </c>
+      <c r="G33">
+        <v>4</v>
+      </c>
+      <c r="H33">
         <v>2021</v>
       </c>
-      <c r="G33" t="str">
-        <v>الولايات المتحدة</v>
-      </c>
-      <c r="H33" t="str">
-        <v>مركز إسعاف كفرسوسة</v>
-      </c>
       <c r="I33" t="str">
-        <v>يُستخدم للطوابق الضيقة والأدراج</v>
+        <v>ألمانيا</v>
+      </c>
+      <c r="J33" t="str">
+        <v>وحدة العناية المركزة</v>
+      </c>
+      <c r="K33" t="str">
+        <v/>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>لوح척추 (척추판) تثبيت척추</v>
+        <v>جهاز الموجات فوق الصوتية (Ultrasound) محمول</v>
       </c>
       <c r="B34" t="str">
-        <v>معدات التثبيت</v>
+        <v>جهاز تشخيص</v>
       </c>
       <c r="C34" t="str">
-        <v>Ferno Model 71</v>
+        <v>GE LOGIQ e R8</v>
       </c>
       <c r="D34" t="str">
-        <v>SN-SPI-001</v>
+        <v>GE-US-2020-01</v>
       </c>
       <c r="E34" t="str">
         <v>جيدة</v>
       </c>
       <c r="F34">
-        <v>2022</v>
-      </c>
-      <c r="G34" t="str">
-        <v>الولايات المتحدة</v>
-      </c>
-      <c r="H34" t="str">
-        <v>مركز الإسعاف المركزي</v>
+        <v>1</v>
+      </c>
+      <c r="G34">
+        <v>1</v>
+      </c>
+      <c r="H34">
+        <v>2020</v>
       </c>
       <c r="I34" t="str">
-        <v>مع 4 أحزمة</v>
+        <v>الولايات المتحدة</v>
+      </c>
+      <c r="J34" t="str">
+        <v>قسم الطوارئ</v>
+      </c>
+      <c r="K34" t="str">
+        <v>تحديث البرنامج v3.2.1 — ضمان حتى 2027</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>لوح척추 (척추판) تثبيت척추</v>
+        <v>جهاز الموجات فوق الصوتية (Ultrasound) ثابت</v>
       </c>
       <c r="B35" t="str">
-        <v>معدات التثبيت</v>
+        <v>جهاز تشخيص</v>
       </c>
       <c r="C35" t="str">
-        <v>Ferno Model 71</v>
+        <v>Mindray DC-70</v>
       </c>
       <c r="D35" t="str">
-        <v>SN-SPI-002</v>
+        <v>MR-US-2022-01</v>
       </c>
       <c r="E35" t="str">
         <v>جيدة</v>
       </c>
       <c r="F35">
+        <v>1</v>
+      </c>
+      <c r="G35">
+        <v>1</v>
+      </c>
+      <c r="H35">
         <v>2022</v>
       </c>
-      <c r="G35" t="str">
-        <v>الولايات المتحدة</v>
-      </c>
-      <c r="H35" t="str">
-        <v>مركز إسعاف المزة</v>
-      </c>
       <c r="I35" t="str">
-        <v>مقاس 76×40 سم — مع مقابض جانبية</v>
+        <v>الصين</v>
+      </c>
+      <c r="J35" t="str">
+        <v>غرفة الأشعة</v>
+      </c>
+      <c r="K35" t="str">
+        <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>طوق عنق طبي قابل للتعديل مجموعة</v>
+        <v>منظار أذن وعين (Otoscope/Ophthalmoscope)</v>
       </c>
       <c r="B36" t="str">
-        <v>معدات التثبيت</v>
+        <v>جهاز تشخيص</v>
       </c>
       <c r="C36" t="str">
-        <v>Ambu Perfit ACE</v>
+        <v>Welch Allyn 3.5V</v>
       </c>
       <c r="D36" t="str">
-        <v>SN-COL-001</v>
+        <v/>
       </c>
       <c r="E36" t="str">
         <v>جيدة</v>
       </c>
       <c r="F36">
-        <v>2022</v>
-      </c>
-      <c r="G36" t="str">
-        <v>الدنمارك</v>
-      </c>
-      <c r="H36" t="str">
-        <v>مركز الإسعاف المركزي</v>
+        <v>5</v>
+      </c>
+      <c r="G36">
+        <v>2</v>
+      </c>
+      <c r="H36">
+        <v>2021</v>
       </c>
       <c r="I36" t="str">
-        <v>4 مقاسات في المجموعة</v>
+        <v>الولايات المتحدة</v>
+      </c>
+      <c r="J36" t="str">
+        <v>غرفة الكشف</v>
+      </c>
+      <c r="K36" t="str">
+        <v>مجموعة شاملة — حقيبة جلدية</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>حقيبة طوارئ ظهر كاملة</v>
+        <v>منظار حنجرة (Laryngoscope) مع مجموعة ألسنة</v>
       </c>
       <c r="B37" t="str">
-        <v>حقائب الطوارئ</v>
+        <v>جهاز تشخيص</v>
       </c>
       <c r="C37" t="str">
-        <v>Pax Rescue Bag Pro</v>
+        <v>Welch Allyn MacIntosh Set</v>
       </c>
       <c r="D37" t="str">
-        <v>SN-BAG-001</v>
+        <v/>
       </c>
       <c r="E37" t="str">
         <v>جيدة</v>
       </c>
       <c r="F37">
-        <v>2023</v>
-      </c>
-      <c r="G37" t="str">
-        <v>ألمانيا</v>
-      </c>
-      <c r="H37" t="str">
-        <v>مركز الإسعاف المركزي</v>
+        <v>6</v>
+      </c>
+      <c r="G37">
+        <v>2</v>
+      </c>
+      <c r="H37">
+        <v>2022</v>
       </c>
       <c r="I37" t="str">
-        <v>مجهزة بالكامل</v>
+        <v>الولايات المتحدة</v>
+      </c>
+      <c r="J37" t="str">
+        <v>مخزن الطوارئ</v>
+      </c>
+      <c r="K37" t="str">
+        <v>مقاسات 0-4 — تعقيم بعد كل استخدام</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>حقيبة طوارئ ظهر كاملة</v>
+        <v>جهاز تعقيم بالبخار (Autoclave)</v>
       </c>
       <c r="B38" t="str">
-        <v>حقائب الطوارئ</v>
+        <v>جهاز تعقيم</v>
       </c>
       <c r="C38" t="str">
-        <v>Pax Rescue Bag Pro</v>
+        <v>Tuttnauer 2540M</v>
       </c>
       <c r="D38" t="str">
-        <v>SN-BAG-002</v>
+        <v>TUT-AUT-001</v>
       </c>
       <c r="E38" t="str">
         <v>جيدة</v>
       </c>
       <c r="F38">
-        <v>2022</v>
-      </c>
-      <c r="G38" t="str">
-        <v>ألمانيا</v>
-      </c>
-      <c r="H38" t="str">
-        <v>مركز إسعاف المزة</v>
+        <v>2</v>
+      </c>
+      <c r="G38">
+        <v>1</v>
+      </c>
+      <c r="H38">
+        <v>2019</v>
       </c>
       <c r="I38" t="str">
-        <v>مقاومة للماء — تحمل 40 لتر</v>
+        <v>إسرائيل</v>
+      </c>
+      <c r="J38" t="str">
+        <v>وحدة التعقيم المركزية</v>
+      </c>
+      <c r="K38" t="str">
+        <v>صيانة دورية — فلتر مياه شهري</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>حقيبة إسعافات أولية ميدانية</v>
+        <v>جهاز تعقيم بالأشعة فوق البنفسجية (UV Sterilizer)</v>
       </c>
       <c r="B39" t="str">
-        <v>حقائب الطوارئ</v>
+        <v>جهاز تعقيم</v>
       </c>
       <c r="C39" t="str">
-        <v>Bound Tree Trauma Bag</v>
+        <v>Philips TUV 30W</v>
       </c>
       <c r="D39" t="str">
-        <v>SN-FAK-001</v>
+        <v/>
       </c>
       <c r="E39" t="str">
         <v>جيدة</v>
       </c>
       <c r="F39">
-        <v>2022</v>
-      </c>
-      <c r="G39" t="str">
-        <v>الولايات المتحدة</v>
-      </c>
-      <c r="H39" t="str">
-        <v>مركز إسعاف ركن الدين</v>
+        <v>5</v>
+      </c>
+      <c r="G39">
+        <v>2</v>
+      </c>
+      <c r="H39">
+        <v>2023</v>
       </c>
       <c r="I39" t="str">
-        <v>بكل مستلزمات الإنعاش الأساسية</v>
+        <v>هولندا</v>
+      </c>
+      <c r="J39" t="str">
+        <v>الغرف والمكاتب</v>
+      </c>
+      <c r="K39" t="str">
+        <v>لا يُستخدم بوجود البشر</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>حقيبة إسعافات أولية ميدانية</v>
+        <v>غسالة معقمة للأدوات (Washer Disinfector)</v>
       </c>
       <c r="B40" t="str">
-        <v>حقائب الطوارئ</v>
+        <v>جهاز تعقيم</v>
       </c>
       <c r="C40" t="str">
-        <v>Bound Tree Trauma Bag</v>
+        <v>Miele PG 8528</v>
       </c>
       <c r="D40" t="str">
-        <v>SN-FAK-002</v>
+        <v>MIE-WD-2020-01</v>
       </c>
       <c r="E40" t="str">
-        <v>تحتاج فحص</v>
+        <v>جيدة</v>
       </c>
       <c r="F40">
+        <v>1</v>
+      </c>
+      <c r="G40">
+        <v>1</v>
+      </c>
+      <c r="H40">
         <v>2020</v>
       </c>
-      <c r="G40" t="str">
-        <v>الولايات المتحدة</v>
-      </c>
-      <c r="H40" t="str">
-        <v>مركز إسعاف الميدان</v>
-      </c>
       <c r="I40" t="str">
-        <v>يلزم تجديد المحتويات</v>
+        <v>ألمانيا</v>
+      </c>
+      <c r="J40" t="str">
+        <v>وحدة التعقيم المركزية</v>
+      </c>
+      <c r="K40" t="str">
+        <v>برنامج 93° C — مرخصة للأدوات الجراحية</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>مضخة حقن وريدي إلكترونية</v>
+        <v>طاولة كشف طبية قابلة للتعديل</v>
       </c>
       <c r="B41" t="str">
-        <v>أجهزة التسريب</v>
+        <v>أثاث طبي</v>
       </c>
       <c r="C41" t="str">
-        <v>Fresenius Kabi Agilia</v>
+        <v>Hausmann 4790</v>
       </c>
       <c r="D41" t="str">
-        <v>SN-PMP-001</v>
+        <v/>
       </c>
       <c r="E41" t="str">
         <v>جيدة</v>
       </c>
       <c r="F41">
-        <v>2022</v>
-      </c>
-      <c r="G41" t="str">
-        <v>ألمانيا</v>
-      </c>
-      <c r="H41" t="str">
-        <v>مركز الإسعاف المركزي</v>
+        <v>6</v>
+      </c>
+      <c r="G41">
+        <v>3</v>
+      </c>
+      <c r="H41">
+        <v>2018</v>
       </c>
       <c r="I41" t="str">
-        <v>دقة ±2% — إنذار انتهاء الكيس</v>
+        <v>الولايات المتحدة</v>
+      </c>
+      <c r="J41" t="str">
+        <v>غرف الكشف</v>
+      </c>
+      <c r="K41" t="str">
+        <v/>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>مضخة حقن وريدي إلكترونية</v>
+        <v>خزانة أدوية ذات قفل</v>
       </c>
       <c r="B42" t="str">
-        <v>أجهزة التسريب</v>
+        <v>أثاث طبي</v>
       </c>
       <c r="C42" t="str">
-        <v>Fresenius Kabi Agilia</v>
+        <v>Midmark 7000</v>
       </c>
       <c r="D42" t="str">
-        <v>SN-PMP-002</v>
+        <v/>
       </c>
       <c r="E42" t="str">
-        <v>في الصيانة</v>
+        <v>جيدة</v>
       </c>
       <c r="F42">
+        <v>4</v>
+      </c>
+      <c r="G42">
+        <v>2</v>
+      </c>
+      <c r="H42">
         <v>2020</v>
       </c>
-      <c r="G42" t="str">
-        <v>ألمانيا</v>
-      </c>
-      <c r="H42" t="str">
-        <v>ورشة الصيانة</v>
-      </c>
       <c r="I42" t="str">
-        <v>صيانة دورية سنوية</v>
+        <v>الولايات المتحدة</v>
+      </c>
+      <c r="J42" t="str">
+        <v>غرف الطوارئ</v>
+      </c>
+      <c r="K42" t="str">
+        <v>مفتاح احتياطي لدى المدير</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>سماعة طبية تشخيصية ثنائية الجرس</v>
+        <v>ضوء الفحص الطبي (Examination Light)</v>
       </c>
       <c r="B43" t="str">
-        <v>أدوات التشخيص</v>
+        <v>أثاث طبي</v>
       </c>
       <c r="C43" t="str">
-        <v>Littmann Cardiology IV</v>
+        <v>Luxiflex LED 40000</v>
       </c>
       <c r="D43" t="str">
-        <v>SN-STH-001</v>
+        <v/>
       </c>
       <c r="E43" t="str">
         <v>جيدة</v>
       </c>
       <c r="F43">
-        <v>2022</v>
-      </c>
-      <c r="G43" t="str">
-        <v>الولايات المتحدة</v>
-      </c>
-      <c r="H43" t="str">
-        <v>د. أحمد الخطيب</v>
+        <v>5</v>
+      </c>
+      <c r="G43">
+        <v>2</v>
+      </c>
+      <c r="H43">
+        <v>2021</v>
       </c>
       <c r="I43" t="str">
-        <v>مع حساسات ECG، SpO2، NIBP جاهزة</v>
+        <v>ألمانيا</v>
+      </c>
+      <c r="J43" t="str">
+        <v>غرف الكشف</v>
+      </c>
+      <c r="K43" t="str">
+        <v>LED — عمر مصباح +50000 ساعة</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>سماعة طبية تشخيصية ثنائية الجرس</v>
+        <v>حامل محلول وريدي (IV Stand) قابل للتعديل</v>
       </c>
       <c r="B44" t="str">
-        <v>أدوات التشخيص</v>
+        <v>أثاث طبي</v>
       </c>
       <c r="C44" t="str">
-        <v>Littmann Classic III</v>
+        <v>Blickman 8951SC</v>
       </c>
       <c r="D44" t="str">
-        <v>SN-STH-002</v>
+        <v/>
       </c>
       <c r="E44" t="str">
         <v>جيدة</v>
       </c>
       <c r="F44">
-        <v>2021</v>
-      </c>
-      <c r="G44" t="str">
-        <v>الولايات المتحدة</v>
-      </c>
-      <c r="H44" t="str">
-        <v>د. سارة الأحمد</v>
+        <v>20</v>
+      </c>
+      <c r="G44">
+        <v>8</v>
+      </c>
+      <c r="H44">
+        <v>2022</v>
       </c>
       <c r="I44" t="str">
-        <v>نموذج قياسي يُغطي الرقبة والظهر العلوي</v>
+        <v>الولايات المتحدة</v>
+      </c>
+      <c r="J44" t="str">
+        <v>أجنحة المرضى</v>
+      </c>
+      <c r="K44" t="str">
+        <v>5 مشابك — فولاذ مقاوم للصدأ</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>سماعة طبية تشخيصية ثنائية الجرس</v>
+        <v>مرتبة واقية ضد قرح الفراش</v>
       </c>
       <c r="B45" t="str">
-        <v>أدوات التشخيص</v>
+        <v>أثاث طبي</v>
       </c>
       <c r="C45" t="str">
-        <v>Littmann Classic III</v>
+        <v>Harvest Healthcare Supreme</v>
       </c>
       <c r="D45" t="str">
-        <v>SN-STH-003</v>
+        <v/>
       </c>
       <c r="E45" t="str">
         <v>جيدة</v>
       </c>
       <c r="F45">
-        <v>2021</v>
-      </c>
-      <c r="G45" t="str">
-        <v>الولايات المتحدة</v>
-      </c>
-      <c r="H45" t="str">
-        <v>د. محمد الزيدان</v>
+        <v>12</v>
+      </c>
+      <c r="G45">
+        <v>5</v>
+      </c>
+      <c r="H45">
+        <v>2022</v>
       </c>
       <c r="I45" t="str">
-        <v>موديل للأطفال — مقاسات 00 إلى 2</v>
+        <v>المملكة المتحدة</v>
+      </c>
+      <c r="J45" t="str">
+        <v>أجنحة المرضى</v>
+      </c>
+      <c r="K45" t="str">
+        <v>ضغط هواء متناوب</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>جهاز رصد ضغط مستمر NIBP</v>
+        <v>حقيبة إسعاف أولي المتقدمة (Trauma Bag)</v>
       </c>
       <c r="B46" t="str">
-        <v>أجهزة المراقبة</v>
+        <v>معدات إسعافية</v>
       </c>
       <c r="C46" t="str">
-        <v>Welch Allyn ABPM 7100</v>
+        <v>Ferno Infinity Trauma</v>
       </c>
       <c r="D46" t="str">
-        <v>SN-NIBP-001</v>
+        <v/>
       </c>
       <c r="E46" t="str">
         <v>جيدة</v>
       </c>
       <c r="F46">
+        <v>8</v>
+      </c>
+      <c r="G46">
+        <v>3</v>
+      </c>
+      <c r="H46">
         <v>2022</v>
       </c>
-      <c r="G46" t="str">
-        <v>الولايات المتحدة</v>
-      </c>
-      <c r="H46" t="str">
-        <v>مركز الإسعاف المركزي</v>
-      </c>
       <c r="I46" t="str">
-        <v>سماعة طبية أمراض داخلية — معدنية ثقيلة</v>
+        <v>الولايات المتحدة</v>
+      </c>
+      <c r="J46" t="str">
+        <v>سيارات الإسعاف</v>
+      </c>
+      <c r="K46" t="str">
+        <v>تحتوي على: ضمادات، قفازات، مشابك، ملقط</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>مصباح فحص رأسي LED محمول</v>
+        <v>جبيرة هوائية للأطراف (Pneumatic Splint) — مجموعة</v>
       </c>
       <c r="B47" t="str">
-        <v>أدوات الفحص</v>
+        <v>معدات إسعافية</v>
       </c>
       <c r="C47" t="str">
-        <v>Petzl Duo S</v>
+        <v>Hartwell Medical Air Splint</v>
       </c>
       <c r="D47" t="str">
-        <v>SN-HLT-001</v>
+        <v/>
       </c>
       <c r="E47" t="str">
         <v>جيدة</v>
       </c>
       <c r="F47">
-        <v>2022</v>
-      </c>
-      <c r="G47" t="str">
-        <v>فرنسا</v>
-      </c>
-      <c r="H47" t="str">
-        <v>مركز الإسعاف المركزي</v>
+        <v>6</v>
+      </c>
+      <c r="G47">
+        <v>2</v>
+      </c>
+      <c r="H47">
+        <v>2021</v>
       </c>
       <c r="I47" t="str">
-        <v>بطارية تدوم 300 ساعة</v>
+        <v>الولايات المتحدة</v>
+      </c>
+      <c r="J47" t="str">
+        <v>مخزن الطوارئ</v>
+      </c>
+      <c r="K47" t="str">
+        <v>3 مقاسات — كامل/نصف طول للذراع والساق</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>مصباح فحص رأسي LED محمول</v>
+        <v>جهاز ضغط على الجرح (Tourniquet) — Combat Application</v>
       </c>
       <c r="B48" t="str">
-        <v>أدوات الفحص</v>
+        <v>معدات إسعافية</v>
       </c>
       <c r="C48" t="str">
-        <v>Petzl Duo S</v>
+        <v>CAT Gen7</v>
       </c>
       <c r="D48" t="str">
-        <v>SN-HLT-002</v>
+        <v/>
       </c>
       <c r="E48" t="str">
         <v>جيدة</v>
       </c>
       <c r="F48">
-        <v>2022</v>
-      </c>
-      <c r="G48" t="str">
-        <v>فرنسا</v>
-      </c>
-      <c r="H48" t="str">
-        <v>مركز إسعاف المزة</v>
+        <v>25</v>
+      </c>
+      <c r="G48">
+        <v>10</v>
+      </c>
+      <c r="H48">
+        <v>2023</v>
       </c>
       <c r="I48" t="str">
-        <v>شاحن USB مرفق — وزن 98 غرام</v>
+        <v>الولايات المتحدة</v>
+      </c>
+      <c r="J48" t="str">
+        <v>سيارات الإسعاف ومخزن الطوارئ</v>
+      </c>
+      <c r="K48" t="str">
+        <v/>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>مجموعة جبائر هوائية للأطراف</v>
+        <v>بطانية إسعافية حرارية (Emergency Blanket) فويل</v>
       </c>
       <c r="B49" t="str">
-        <v>معدات التثبيت</v>
+        <v>معدات إسعافية</v>
       </c>
       <c r="C49" t="str">
-        <v>Hartwell Medical</v>
+        <v>North American Rescue</v>
       </c>
       <c r="D49" t="str">
-        <v>SN-SPL-001</v>
+        <v/>
       </c>
       <c r="E49" t="str">
         <v>جيدة</v>
       </c>
       <c r="F49">
-        <v>2022</v>
-      </c>
-      <c r="G49" t="str">
-        <v>الولايات المتحدة</v>
-      </c>
-      <c r="H49" t="str">
-        <v>مركز الإسعاف المركزي</v>
+        <v>50</v>
+      </c>
+      <c r="G49">
+        <v>20</v>
+      </c>
+      <c r="H49">
+        <v>2024</v>
       </c>
       <c r="I49" t="str">
-        <v>صغير ومتوسط وكبير</v>
+        <v>الولايات المتحدة</v>
+      </c>
+      <c r="J49" t="str">
+        <v>مخزن الطوارئ</v>
+      </c>
+      <c r="K49" t="str">
+        <v>للاستخدام مرة واحدة — مقاوم للرياح والرطوبة</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>مجموعة جبائر تشكيلية SAM</v>
+        <v>جهاز لاسلكي محمول (Walkie-Talkie) للميدان</v>
       </c>
       <c r="B50" t="str">
-        <v>معدات التثبيت</v>
+        <v>معدات اتصال</v>
       </c>
       <c r="C50" t="str">
-        <v>SAM Medical</v>
+        <v>Motorola DP4400e</v>
       </c>
       <c r="D50" t="str">
-        <v>SN-SAM-001</v>
+        <v>MOT-VHF-101</v>
       </c>
       <c r="E50" t="str">
         <v>جيدة</v>
       </c>
       <c r="F50">
+        <v>10</v>
+      </c>
+      <c r="G50">
+        <v>4</v>
+      </c>
+      <c r="H50">
         <v>2021</v>
       </c>
-      <c r="G50" t="str">
-        <v>الولايات المتحدة</v>
-      </c>
-      <c r="H50" t="str">
-        <v>مركز إسعاف كفرسوسة</v>
-      </c>
       <c r="I50" t="str">
-        <v>جبائر SAM قابلة لإعادة التشكيل عدة مرات</v>
+        <v>الولايات المتحدة</v>
+      </c>
+      <c r="J50" t="str">
+        <v>سيارات الإسعاف</v>
+      </c>
+      <c r="K50" t="str">
+        <v>شبكة VHF — بطارية 12 ساعة</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>ضوء فلاش طوارئ للسيارة</v>
+        <v>جهاز لاسلكي محمول (Walkie-Talkie) للميدان</v>
       </c>
       <c r="B51" t="str">
-        <v>معدات الطوارئ</v>
+        <v>معدات اتصال</v>
       </c>
       <c r="C51" t="str">
-        <v>Federal Signal Vision SLR</v>
+        <v>Motorola DP4400e</v>
       </c>
       <c r="D51" t="str">
-        <v>SN-FLH-001</v>
+        <v>MOT-VHF-102</v>
       </c>
       <c r="E51" t="str">
         <v>جيدة</v>
       </c>
       <c r="F51">
-        <v>2022</v>
-      </c>
-      <c r="G51" t="str">
-        <v>الولايات المتحدة</v>
-      </c>
-      <c r="H51" t="str">
-        <v>سيارة الإسعاف 01</v>
+        <v>10</v>
+      </c>
+      <c r="G51">
+        <v>4</v>
+      </c>
+      <c r="H51">
+        <v>2021</v>
       </c>
       <c r="I51" t="str">
-        <v>مزود بمصباح LED و3 أوضاع إضاءة</v>
+        <v>الولايات المتحدة</v>
+      </c>
+      <c r="J51" t="str">
+        <v>غرفة العمليات</v>
+      </c>
+      <c r="K51" t="str">
+        <v>احتياطي</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>مكبر صوت طوارئ</v>
+        <v>خوذة واقية للمسعفين</v>
       </c>
       <c r="B52" t="str">
-        <v>معدات الطوارئ</v>
+        <v>معدات حماية</v>
       </c>
       <c r="C52" t="str">
-        <v>Federal Signal PA640</v>
+        <v>MSA V-Gard 500</v>
       </c>
       <c r="D52" t="str">
-        <v>SN-SRN-001</v>
+        <v/>
       </c>
       <c r="E52" t="str">
         <v>جيدة</v>
       </c>
       <c r="F52">
-        <v>2021</v>
-      </c>
-      <c r="G52" t="str">
-        <v>الولايات المتحدة</v>
-      </c>
-      <c r="H52" t="str">
-        <v>سيارة الإسعاف 01</v>
+        <v>15</v>
+      </c>
+      <c r="G52">
+        <v>6</v>
+      </c>
+      <c r="H52">
+        <v>2022</v>
       </c>
       <c r="I52" t="str">
-        <v>مكبر + شريط LED أصفر للتحذير</v>
+        <v>الولايات المتحدة</v>
+      </c>
+      <c r="J52" t="str">
+        <v>مخزن التجهيزات الشخصية</v>
+      </c>
+      <c r="K52" t="str">
+        <v>درجة EN397 — تفتيش سنوي</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>جهاز راديو اتصال لاسلكي</v>
+        <v>سترة واقية عاكسة للمسعفين</v>
       </c>
       <c r="B53" t="str">
-        <v>معدات الاتصال</v>
+        <v>معدات حماية</v>
       </c>
       <c r="C53" t="str">
-        <v>Motorola APX 6000</v>
+        <v>Portwest HiVis</v>
       </c>
       <c r="D53" t="str">
-        <v>SN-RAD-001</v>
+        <v/>
       </c>
       <c r="E53" t="str">
         <v>جيدة</v>
       </c>
       <c r="F53">
-        <v>2022</v>
-      </c>
-      <c r="G53" t="str">
-        <v>الولايات المتحدة</v>
-      </c>
-      <c r="H53" t="str">
-        <v>مركز الإسعاف المركزي</v>
+        <v>20</v>
+      </c>
+      <c r="G53">
+        <v>8</v>
+      </c>
+      <c r="H53">
+        <v>2023</v>
       </c>
       <c r="I53" t="str">
-        <v>شبكة تشفير متقدمة</v>
+        <v>إيرلندا</v>
+      </c>
+      <c r="J53" t="str">
+        <v>مخزن التجهيزات الشخصية</v>
+      </c>
+      <c r="K53" t="str">
+        <v>فئة 2 — مقاس XL</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>جهاز راديو اتصال لاسلكي</v>
+        <v>مصباح يدوي قوي للميدان</v>
       </c>
       <c r="B54" t="str">
-        <v>معدات الاتصال</v>
+        <v>معدات حماية</v>
       </c>
       <c r="C54" t="str">
-        <v>Motorola APX 6000</v>
+        <v>Streamlight Stinger DS LED</v>
       </c>
       <c r="D54" t="str">
-        <v>SN-RAD-002</v>
+        <v/>
       </c>
       <c r="E54" t="str">
         <v>جيدة</v>
       </c>
       <c r="F54">
+        <v>12</v>
+      </c>
+      <c r="G54">
+        <v>5</v>
+      </c>
+      <c r="H54">
         <v>2022</v>
       </c>
-      <c r="G54" t="str">
-        <v>الولايات المتحدة</v>
-      </c>
-      <c r="H54" t="str">
-        <v>مركز إسعاف المزة</v>
-      </c>
       <c r="I54" t="str">
-        <v>بطارية تدوم 18 ساعة — شبكة UHF مشفرة</v>
+        <v>الولايات المتحدة</v>
+      </c>
+      <c r="J54" t="str">
+        <v>سيارات الإسعاف</v>
+      </c>
+      <c r="K54" t="str">
+        <v>يُشحن من ولاعة السيارة</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>جهاز راديو اتصال لاسلكي</v>
+        <v>جهاز قياس ثاني أكسيد الكربون الزفيري (Capnograph)</v>
       </c>
       <c r="B55" t="str">
-        <v>معدات الاتصال</v>
+        <v>جهاز تشخيص</v>
       </c>
       <c r="C55" t="str">
-        <v>Kenwood TK-3401D</v>
+        <v>Oridion Microstream CO2</v>
       </c>
       <c r="D55" t="str">
-        <v>SN-RAD-003</v>
+        <v>ORI-CAP-0012</v>
       </c>
       <c r="E55" t="str">
-        <v>مستهلكة</v>
+        <v>جيدة</v>
       </c>
       <c r="F55">
-        <v>2017</v>
-      </c>
-      <c r="G55" t="str">
-        <v>اليابان</v>
-      </c>
-      <c r="H55" t="str">
-        <v>مستودع التخلص</v>
+        <v>3</v>
+      </c>
+      <c r="G55">
+        <v>1</v>
+      </c>
+      <c r="H55">
+        <v>2021</v>
       </c>
       <c r="I55" t="str">
-        <v>انتهى عمرها الافتراضي</v>
+        <v>إسرائيل</v>
+      </c>
+      <c r="J55" t="str">
+        <v>سيارة إسعاف 1</v>
+      </c>
+      <c r="K55" t="str">
+        <v>يستلزم خراطيم مخصصة للاستخدام مرة واحدة</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>حقيبة إسعاف الحروق المتخصصة</v>
+        <v>منظار للتنبيب الصعب (Video Laryngoscope)</v>
       </c>
       <c r="B56" t="str">
-        <v>حقائب الطوارئ</v>
+        <v>جهاز تشخيص</v>
       </c>
       <c r="C56" t="str">
-        <v>H&amp;H Medical Burns Kit</v>
+        <v>McGrath MAC</v>
       </c>
       <c r="D56" t="str">
-        <v>SN-BRN-001</v>
+        <v>MG-VL-0003</v>
       </c>
       <c r="E56" t="str">
         <v>جيدة</v>
       </c>
       <c r="F56">
+        <v>2</v>
+      </c>
+      <c r="G56">
+        <v>1</v>
+      </c>
+      <c r="H56">
         <v>2022</v>
       </c>
-      <c r="G56" t="str">
-        <v>الولايات المتحدة</v>
-      </c>
-      <c r="H56" t="str">
-        <v>مركز الإسعاف المركزي</v>
-      </c>
       <c r="I56" t="str">
-        <v>جهاز مستهلك — يلزم إصدار أمر إتلاف</v>
+        <v>المملكة المتحدة</v>
+      </c>
+      <c r="J56" t="str">
+        <v>غرفة العمليات 1</v>
+      </c>
+      <c r="K56" t="str">
+        <v>شاشة LCD 2.5 بوصة — يستلزم ألسنة معقمة</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>جهاز تدفئة المحاليل الوريدية</v>
+        <v>جهاز رصد درجة حرارة المريض الأساسية</v>
       </c>
       <c r="B57" t="str">
-        <v>أجهزة التسريب</v>
+        <v>جهاز قياس</v>
       </c>
       <c r="C57" t="str">
-        <v>3M Ranger 245</v>
+        <v>Welch Allyn SureTemp 692</v>
       </c>
       <c r="D57" t="str">
-        <v>SN-FLD-001</v>
+        <v>WA-TEMP-0044</v>
       </c>
       <c r="E57" t="str">
         <v>جيدة</v>
       </c>
       <c r="F57">
-        <v>2021</v>
-      </c>
-      <c r="G57" t="str">
-        <v>الولايات المتحدة</v>
-      </c>
-      <c r="H57" t="str">
-        <v>مركز الإسعاف المركزي</v>
+        <v>4</v>
+      </c>
+      <c r="G57">
+        <v>2</v>
+      </c>
+      <c r="H57">
+        <v>2020</v>
       </c>
       <c r="I57" t="str">
-        <v>محلول هيدروجيل ملطف — بدون كحول</v>
+        <v>الولايات المتحدة</v>
+      </c>
+      <c r="J57" t="str">
+        <v>غرف الكشف</v>
+      </c>
+      <c r="K57" t="str">
+        <v>يقيس درجة حرارة المريض خلال 10 ثوانٍ</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>مجموعة تثبيت척추 الرأس والرقبة</v>
+        <v>مضخة شفط الجرح (Wound VAC)</v>
       </c>
       <c r="B58" t="str">
-        <v>معدات التثبيت</v>
+        <v>جهاز علاجي</v>
       </c>
       <c r="C58" t="str">
-        <v>Laerdal Head Immobilizer</v>
+        <v>KCI ActiV.A.C.</v>
       </c>
       <c r="D58" t="str">
-        <v>SN-HIM-001</v>
+        <v>KCI-VAC-0007</v>
       </c>
       <c r="E58" t="str">
         <v>جيدة</v>
       </c>
       <c r="F58">
-        <v>2022</v>
-      </c>
-      <c r="G58" t="str">
-        <v>النرويج</v>
-      </c>
-      <c r="H58" t="str">
-        <v>مركز الإسعاف المركزي</v>
+        <v>2</v>
+      </c>
+      <c r="G58">
+        <v>1</v>
+      </c>
+      <c r="H58">
+        <v>2021</v>
       </c>
       <c r="I58" t="str">
-        <v>درجة حرارة تعمل من 10 إلى 45 مئوية</v>
+        <v>الولايات المتحدة</v>
+      </c>
+      <c r="J58" t="str">
+        <v>وحدة الجراحة</v>
+      </c>
+      <c r="K58" t="str">
+        <v>ضمادات مخصصة — للاستخدام مرة واحدة</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>طقم جبيرة تراكشن للساق</v>
+        <v>جهاز تسخين السوائل الوريدية (Fluid Warmer)</v>
       </c>
       <c r="B59" t="str">
-        <v>معدات التثبيت</v>
+        <v>جهاز علاجي</v>
       </c>
       <c r="C59" t="str">
-        <v>Sager Emergency Traction</v>
+        <v>Smiths Medical Level 1</v>
       </c>
       <c r="D59" t="str">
-        <v>SN-TRC-001</v>
+        <v>SM-FW-0018</v>
       </c>
       <c r="E59" t="str">
         <v>جيدة</v>
       </c>
       <c r="F59">
-        <v>2021</v>
-      </c>
-      <c r="G59" t="str">
-        <v>الولايات المتحدة</v>
-      </c>
-      <c r="H59" t="str">
-        <v>مركز الإسعاف المركزي</v>
+        <v>3</v>
+      </c>
+      <c r="G59">
+        <v>1</v>
+      </c>
+      <c r="H59">
+        <v>2022</v>
       </c>
       <c r="I59" t="str">
-        <v>رأس قابل للدوران 360 درجة</v>
+        <v>الولايات المتحدة</v>
+      </c>
+      <c r="J59" t="str">
+        <v>غرفة العمليات</v>
+      </c>
+      <c r="K59" t="str">
+        <v>يرفع درجة حرارة المحلول لـ 41° C</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>حاضنة نقل أطفال حديثي الولادة</v>
+        <v>جهاز كسر عظمة القص للإنعاش (LUCAS 3)</v>
       </c>
       <c r="B60" t="str">
-        <v>أجهزة التخصصية</v>
+        <v>جهاز إنعاش</v>
       </c>
       <c r="C60" t="str">
-        <v>GE Giraffe OmniBed</v>
+        <v>Stryker LUCAS 3</v>
       </c>
       <c r="D60" t="str">
-        <v>SN-INC-001</v>
+        <v>STR-LUC-0002</v>
       </c>
       <c r="E60" t="str">
         <v>جيدة</v>
       </c>
       <c r="F60">
+        <v>2</v>
+      </c>
+      <c r="G60">
+        <v>1</v>
+      </c>
+      <c r="H60">
         <v>2023</v>
       </c>
-      <c r="G60" t="str">
-        <v>الولايات المتحدة</v>
-      </c>
-      <c r="H60" t="str">
-        <v>مركز الإسعاف المركزي</v>
-      </c>
       <c r="I60" t="str">
-        <v>للنقل الطارئ فقط</v>
+        <v>الولايات المتحدة</v>
+      </c>
+      <c r="J60" t="str">
+        <v>سيارة إسعاف 1</v>
+      </c>
+      <c r="K60" t="str">
+        <v>ضغط آلي على القص — يحرر يدي المسعف</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>مجموعة ولادة طارئة</v>
+        <v>مضخة تصريف الصدر (Chest Drain Pump)</v>
       </c>
       <c r="B61" t="str">
-        <v>معدات التوليد</v>
+        <v>جهاز علاجي</v>
       </c>
       <c r="C61" t="str">
-        <v>Medline Emergency OB Kit</v>
+        <v>Atrium Ocean 3603</v>
       </c>
       <c r="D61" t="str">
-        <v>SN-OBK-001</v>
+        <v>ATR-CDP-0009</v>
       </c>
       <c r="E61" t="str">
         <v>جيدة</v>
       </c>
       <c r="F61">
-        <v>2023</v>
-      </c>
-      <c r="G61" t="str">
-        <v>الولايات المتحدة</v>
-      </c>
-      <c r="H61" t="str">
-        <v>مركز الإسعاف المركزي</v>
+        <v>2</v>
+      </c>
+      <c r="G61">
+        <v>1</v>
+      </c>
+      <c r="H61">
+        <v>2022</v>
       </c>
       <c r="I61" t="str">
-        <v>معقمة ومغلفة</v>
+        <v>الولايات المتحدة</v>
+      </c>
+      <c r="J61" t="str">
+        <v>وحدة الجراحة</v>
+      </c>
+      <c r="K61" t="str">
+        <v>استنزاف الهواء والسوائل من التجويف الجنبي</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I61"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K61"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:B28"/>
   <cols>
-    <col min="1" max="1" width="18.83203125" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" customWidth="1"/>
-    <col min="3" max="3" width="40.83203125" customWidth="1"/>
+    <col min="1" max="1" width="40.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>تعليمات الاستخدام — نموذج استيراد التجهيزات</v>
+        <v>إحصائيات ملف الاختبار</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>العمود</v>
+        <v>المعلومة</v>
       </c>
       <c r="B3" t="str">
-        <v>الوصف</v>
-      </c>
-      <c r="C3" t="str">
-        <v>مطلوب؟</v>
-      </c>
-      <c r="D3" t="str">
-        <v>ملاحظات</v>
+        <v>القيمة</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>الاسم *</v>
-      </c>
-      <c r="B4" t="str">
-        <v>اسم التجهيز أو الجهاز</v>
-      </c>
-      <c r="C4" t="str">
-        <v>نعم</v>
-      </c>
-      <c r="D4" t="str">
-        <v/>
+        <v>إجمالي التجهيزات</v>
+      </c>
+      <c r="B4">
+        <v>60</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>نوع التجهيز</v>
-      </c>
-      <c r="B5" t="str">
-        <v>تصنيف التجهيز</v>
-      </c>
-      <c r="C5" t="str">
-        <v>لا</v>
-      </c>
-      <c r="D5" t="str">
-        <v>مثال: جهاز طوارئ، جهاز مراقبة، أثاث طبي</v>
+        <v>تجهيزات جيدة</v>
+      </c>
+      <c r="B5">
+        <v>57</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>الموديل</v>
-      </c>
-      <c r="B6" t="str">
-        <v>رقم الموديل أو الطراز</v>
-      </c>
-      <c r="C6" t="str">
-        <v>لا</v>
-      </c>
-      <c r="D6" t="str">
-        <v/>
+        <v>تجهيزات تحتاج فحص</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>الرقم التسلسلي</v>
-      </c>
-      <c r="B7" t="str">
-        <v>الرقم التسلسلي الفريد</v>
-      </c>
-      <c r="C7" t="str">
-        <v>لا</v>
-      </c>
-      <c r="D7" t="str">
-        <v>يجب أن يكون فريداً إذا أُدخل</v>
+        <v>تجهيزات في الصيانة</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>الحالة</v>
-      </c>
-      <c r="B8" t="str">
-        <v>حالة التجهيز الحالية</v>
-      </c>
-      <c r="C8" t="str">
-        <v>لا</v>
-      </c>
-      <c r="D8" t="str">
-        <v>القيم المقبولة: جيدة — في الصيانة — معطلة — مستهلكة — تحتاج فحص</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>سنة الصنع</v>
-      </c>
-      <c r="B9" t="str">
-        <v>السنة الميلادية للتصنيع</v>
-      </c>
-      <c r="C9" t="str">
-        <v>لا</v>
-      </c>
-      <c r="D9" t="str">
-        <v>رقم بين 1900 و2100</v>
+        <v>تجهيزات معطلة</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>بلد المنشأ</v>
-      </c>
-      <c r="B10" t="str">
-        <v>بلد التصنيع</v>
-      </c>
-      <c r="C10" t="str">
-        <v>لا</v>
-      </c>
-      <c r="D10" t="str">
-        <v/>
+        <v>تجهيزات بكمية ≥ 10 قطعة</v>
+      </c>
+      <c r="B10">
+        <v>20</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>الحائز الحالي</v>
-      </c>
-      <c r="B11" t="str">
-        <v>القسم أو الشخص المسؤول</v>
-      </c>
-      <c r="C11" t="str">
-        <v>لا</v>
-      </c>
-      <c r="D11" t="str">
-        <v/>
+        <v>تجهيزات بكمية ≤ 3 قطع</v>
+      </c>
+      <c r="B11">
+        <v>16</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>ملاحظات</v>
-      </c>
-      <c r="B12" t="str">
-        <v>أي ملاحظات إضافية</v>
-      </c>
-      <c r="C12" t="str">
-        <v>لا</v>
-      </c>
-      <c r="D12" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>توزيع بيانات الاختبار (60 تجهيزة):</v>
+        <v>تجهيزات بها حد أدنى (تنبيه)</v>
+      </c>
+      <c r="B12">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>تجهيزات بكمية أقل من الحد الأدنى (نقص!)</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>الحالة</v>
-      </c>
-      <c r="B15" t="str">
-        <v>العدد</v>
-      </c>
-      <c r="C15" t="str">
-        <v>الغرض من الاختبار</v>
+        <v>بلدان الصنع الأكثر شيوعاً</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>جيدة</v>
-      </c>
-      <c r="B16" t="str">
-        <v>50</v>
-      </c>
-      <c r="C16" t="str">
-        <v>الحالة الطبيعية — الأغلبية</v>
+        <v>الولايات المتحدة</v>
+      </c>
+      <c r="B16">
+        <v>32</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>في الصيانة</v>
-      </c>
-      <c r="B17" t="str">
-        <v>4</v>
-      </c>
-      <c r="C17" t="str">
-        <v>اختبار تتبع الأجهزة خارج الخدمة مؤقتاً</v>
+        <v>ألمانيا</v>
+      </c>
+      <c r="B17">
+        <v>9</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>تحتاج فحص</v>
-      </c>
-      <c r="B18" t="str">
+        <v>الصين</v>
+      </c>
+      <c r="B18">
         <v>4</v>
-      </c>
-      <c r="C18" t="str">
-        <v>اختبار التنبيهات والتحذيرات</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>معطلة</v>
-      </c>
-      <c r="B19" t="str">
-        <v>1</v>
-      </c>
-      <c r="C19" t="str">
-        <v>اختبار الأجهزة خارج الخدمة نهائياً</v>
+        <v>هولندا</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>مستهلكة</v>
-      </c>
-      <c r="B20" t="str">
+        <v>النرويج</v>
+      </c>
+      <c r="B20">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>فرنسا</v>
+      </c>
+      <c r="B21">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>إسرائيل</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>المملكة المتحدة</v>
+      </c>
+      <c r="B23">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>الدنمارك</v>
+      </c>
+      <c r="B24">
         <v>1</v>
       </c>
-      <c r="C20" t="str">
-        <v>اختبار إتلاف/شطب الأجهزة</v>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>اليابان</v>
+      </c>
+      <c r="B25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>سويسرا</v>
+      </c>
+      <c r="B26">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>نيوزيلندا</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>إيرلندا</v>
+      </c>
+      <c r="B28">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D20"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B28"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>